<commit_message>
Publish Prague_2021_WC, Prague_2022_WC, Prague_2023_WC, RioDeJaneiro_2018_WCH
</commit_message>
<xml_diff>
--- a/events/Prague_2021_WC/Prague_2021_WC_start.xlsx
+++ b/events/Prague_2021_WC/Prague_2021_WC_start.xlsx
@@ -28085,6 +28085,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X477" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -36398,6 +36403,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X613" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
@@ -39856,6 +39866,11 @@
       <c r="R668" t="inlineStr">
         <is>
           <t>FISEROVA Tereza</t>
+        </is>
+      </c>
+      <c r="X668" t="inlineStr">
+        <is>
+          <t>42016</t>
         </is>
       </c>
     </row>

</xml_diff>